<commit_message>
feat(test): add router_iteratively and CLI case config for iterative tests / 新增 router_iteratively 迭代测试并支持命令行指定用例
Add routing-only 100-run stability test, allow placer_iteratively to accept config via argv, default to case1, and update case1 connections plus docs. / 新增仅布线 100 轮稳定性测试，placer_iteratively 支持 argv 指定用例且默认 case1，并更新 case1 连接与文档。

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/test/config/case1/case1.xlsx
+++ b/test/config/case1/case1.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="10455" activeTab="1"/>
+    <workbookView windowWidth="24900" windowHeight="13660" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="muyan信号与bumpbank对应关系" sheetId="2" r:id="rId1"/>
@@ -12,25 +12,12 @@
     <sheet name="外部IO说明" sheetId="4" r:id="rId3"/>
     <sheet name="muyan与tob对应关系" sheetId="5" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="484">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="363">
   <si>
     <t>序号</t>
   </si>
@@ -791,388 +778,46 @@
     <t>xinzhai_spi_s_din_1</t>
   </si>
   <si>
-    <t>muyan_1_s_tx_flit_b0</t>
-  </si>
-  <si>
-    <t>muyan_0_m_rx_flit_b0</t>
-  </si>
-  <si>
-    <t>muyan_1_s_tx_flit_b1</t>
-  </si>
-  <si>
-    <t>muyan_0_m_rx_flit_b1</t>
-  </si>
-  <si>
-    <t>muyan_1_s_tx_flit_b2</t>
-  </si>
-  <si>
-    <t>muyan_0_m_rx_flit_b2</t>
-  </si>
-  <si>
-    <t>muyan_1_s_tx_flit_b3</t>
-  </si>
-  <si>
-    <t>muyan_0_m_rx_flit_b3</t>
-  </si>
-  <si>
-    <t>muyan_1_s_tx_flit_b4</t>
-  </si>
-  <si>
-    <t>muyan_0_m_rx_flit_b4</t>
-  </si>
-  <si>
-    <t>muyan_1_s_tx_flit_b5</t>
-  </si>
-  <si>
-    <t>muyan_0_m_rx_flit_b5</t>
-  </si>
-  <si>
-    <t>muyan_1_s_tx_flit_b6</t>
-  </si>
-  <si>
-    <t>muyan_0_m_rx_flit_b6</t>
-  </si>
-  <si>
-    <t>muyan_1_s_tx_flit_b7</t>
-  </si>
-  <si>
-    <t>muyan_0_m_rx_flit_b7</t>
-  </si>
-  <si>
-    <t>muyan_1_s_tx_rplyPkgID</t>
-  </si>
-  <si>
-    <t>muyan_0_m_rx_rplyPkgID</t>
-  </si>
-  <si>
-    <t>muyan_1_s_tx_crdtARW_free</t>
-  </si>
-  <si>
-    <t>muyan_0_m_rx_crdtARW_free</t>
-  </si>
-  <si>
-    <t>muyan_1_s_tx_clk</t>
-  </si>
-  <si>
-    <t>muyan_0_m_rx_clk</t>
-  </si>
-  <si>
-    <t>muyan_1_s_tx_flit_vld</t>
-  </si>
-  <si>
-    <t>muyan_0_m_rx_flit_vld</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_flit_b0</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_flit_b0</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_flit_b1</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_flit_b1</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_flit_b2</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_flit_b2</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_flit_b3</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_flit_b3</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_flit_b4</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_flit_b4</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_flit_b5</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_flit_b5</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_flit_b6</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_flit_b6</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_flit_b7</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_flit_b7</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_flit_b8</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_flit_b8</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_flit_b9</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_flit_b9</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_flit_b10</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_flit_b10</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_flit_b11</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_flit_b11</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_flit_b12</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_flit_b12</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_flit_b13</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_flit_b13</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_flit_b14</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_flit_b14</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_flit_b15</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_flit_b15</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_rplyPkgID</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_rplyPkgID</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_crdtRB_free</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_crdtRB_free</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_clk</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_clk</t>
-  </si>
-  <si>
-    <t>muyan_0_m_tx_flit_vld</t>
-  </si>
-  <si>
-    <t>muyan_1_s_rx_vld</t>
-  </si>
-  <si>
-    <t>muyan_0_s_tx_flit_b0</t>
-  </si>
-  <si>
-    <t>muyan_1_m_rx_flit_b0</t>
-  </si>
-  <si>
-    <t>muyan_0_s_tx_flit_b1</t>
-  </si>
-  <si>
-    <t>muyan_1_m_rx_flit_b1</t>
-  </si>
-  <si>
-    <t>muyan_0_s_tx_flit_b2</t>
-  </si>
-  <si>
-    <t>muyan_1_m_rx_flit_b2</t>
-  </si>
-  <si>
-    <t>muyan_0_s_tx_flit_b3</t>
-  </si>
-  <si>
-    <t>muyan_1_m_rx_flit_b3</t>
-  </si>
-  <si>
-    <t>muyan_0_s_tx_flit_b4</t>
-  </si>
-  <si>
-    <t>muyan_1_m_rx_flit_b4</t>
-  </si>
-  <si>
-    <t>muyan_0_s_tx_flit_b5</t>
-  </si>
-  <si>
-    <t>muyan_1_m_rx_flit_b5</t>
-  </si>
-  <si>
-    <t>muyan_0_s_tx_flit_b6</t>
-  </si>
-  <si>
-    <t>muyan_1_m_rx_flit_b6</t>
-  </si>
-  <si>
-    <t>muyan_0_s_tx_flit_b7</t>
-  </si>
-  <si>
-    <t>muyan_1_m_rx_flit_b7</t>
-  </si>
-  <si>
-    <t>muyan_0_s_tx_rplyPkgID</t>
-  </si>
-  <si>
-    <t>muyan_1_m_rx_rplyPkgID</t>
-  </si>
-  <si>
-    <t>muyan_0_s_tx_crdtARW_free</t>
-  </si>
-  <si>
-    <t>muyan_1_m_rx_crdtARW_free</t>
-  </si>
-  <si>
-    <t>muyan_0_s_tx_clk</t>
-  </si>
-  <si>
-    <t>muyan_1_m_rx_clk</t>
-  </si>
-  <si>
-    <t>muyan_0_s_tx_flit_vld</t>
-  </si>
-  <si>
-    <t>muyan_1_m_rx_flit_vld</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_flit_b0</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_flit_b0</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_flit_b1</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_flit_b1</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_flit_b2</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_flit_b2</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_flit_b3</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_flit_b3</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_flit_b4</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_flit_b4</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_flit_b5</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_flit_b5</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_flit_b6</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_flit_b6</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_flit_b7</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_flit_b7</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_flit_b8</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_flit_b8</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_flit_b9</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_flit_b9</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_flit_b10</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_flit_b10</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_flit_b11</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_flit_b11</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_flit_b12</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_flit_b12</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_flit_b13</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_flit_b13</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_flit_b14</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_flit_b14</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_flit_b15</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_flit_b15</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_rplyPkgID</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_rplyPkgID</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_crdtRB_free</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_crdtRB_free</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_clk</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_clk</t>
-  </si>
-  <si>
-    <t>muyan_1_m_tx_flit_vld</t>
-  </si>
-  <si>
-    <t>muyan_0_s_rx_vld</t>
+    <t>xinzhai_jtag_trstn</t>
+  </si>
+  <si>
+    <t>muyan_0_jtag_trstn</t>
+  </si>
+  <si>
+    <t>xinzhai_jtag_tdi</t>
+  </si>
+  <si>
+    <t>muyan_0_jtag_tdi</t>
+  </si>
+  <si>
+    <t>xinzhai_jtag_tck</t>
+  </si>
+  <si>
+    <t>muyan_0_jtag_tck</t>
+  </si>
+  <si>
+    <t>xinzhai_jtag_tms</t>
+  </si>
+  <si>
+    <t>muyan_0_jtag_tms</t>
+  </si>
+  <si>
+    <t>muyan_0_jtag_tdo</t>
+  </si>
+  <si>
+    <t>xinzhai_jtag_tdo</t>
+  </si>
+  <si>
+    <t>xinzhai_uart_txd</t>
+  </si>
+  <si>
+    <t>muyan_0_uart_rxd</t>
+  </si>
+  <si>
+    <t>muyan_0_uart_txd</t>
+  </si>
+  <si>
+    <t>xinzhai_uart_rxd</t>
   </si>
   <si>
     <t>0 0 5</t>
@@ -1188,27 +833,6 @@
   </si>
   <si>
     <t>xinzhai_spi_mosi</t>
-  </si>
-  <si>
-    <t>xinzhai_jtag_trstn</t>
-  </si>
-  <si>
-    <t>xinzhai_jtag_tdi</t>
-  </si>
-  <si>
-    <t>xinzhai_jtag_tck</t>
-  </si>
-  <si>
-    <t>xinzhai_jtag_tms</t>
-  </si>
-  <si>
-    <t>xinzhai_uart_txd</t>
-  </si>
-  <si>
-    <t>xinzhai_jtag_tdo</t>
-  </si>
-  <si>
-    <t>xinzhai_uart_rxd</t>
   </si>
   <si>
     <t>xinzhai_spi_s_sck_2</t>
@@ -1487,12 +1111,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -1513,7 +1137,21 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
-      <charset val="134"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="等线"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1525,16 +1163,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color theme="3"/>
       <name val="等线"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF006100"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1548,11 +1186,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
       <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
+      <color theme="1"/>
       <name val="等线"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1574,14 +1211,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color rgb="FFFA7D00"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1589,15 +1219,22 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color theme="1"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <u/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF800080"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1612,7 +1249,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FFFF0000"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1620,21 +1257,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
+      <color rgb="FF3F3F3F"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1648,14 +1271,15 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FFFA7D00"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <i/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF7F7F7F"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1676,7 +1300,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1688,7 +1318,109 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1700,19 +1432,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1724,139 +1474,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1911,6 +1535,15 @@
     </border>
     <border>
       <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color auto="1"/>
       </right>
@@ -1931,7 +1564,9 @@
     </border>
     <border>
       <left/>
-      <right/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
       <bottom style="thin">
         <color auto="1"/>
@@ -1939,13 +1574,26 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
+      <right/>
       <top/>
-      <bottom style="thin">
-        <color auto="1"/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1976,24 +1624,26 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
       </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
       </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -2013,21 +1663,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
@@ -2036,162 +1671,151 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="24" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="11" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -2211,10 +1835,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2246,54 +1870,54 @@
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="1" builtinId="52"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="2" builtinId="42"/>
+    <cellStyle name="强调文字颜色 4" xfId="3" builtinId="41"/>
+    <cellStyle name="输入" xfId="4" builtinId="20"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="5" builtinId="39"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="6" builtinId="38"/>
+    <cellStyle name="货币" xfId="7" builtinId="4"/>
+    <cellStyle name="强调文字颜色 3" xfId="8" builtinId="37"/>
+    <cellStyle name="百分比" xfId="9" builtinId="5"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="10" builtinId="36"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="11" builtinId="48"/>
+    <cellStyle name="强调文字颜色 2" xfId="12" builtinId="33"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="13" builtinId="32"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="14" builtinId="44"/>
+    <cellStyle name="计算" xfId="15" builtinId="22"/>
+    <cellStyle name="强调文字颜色 1" xfId="16" builtinId="29"/>
+    <cellStyle name="适中" xfId="17" builtinId="28"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="18" builtinId="46"/>
+    <cellStyle name="好" xfId="19" builtinId="26"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="20" builtinId="30"/>
     <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="差" xfId="22" builtinId="27"/>
+    <cellStyle name="检查单元格" xfId="23" builtinId="23"/>
+    <cellStyle name="输出" xfId="24" builtinId="21"/>
+    <cellStyle name="标题 1" xfId="25" builtinId="16"/>
+    <cellStyle name="解释性文本" xfId="26" builtinId="53"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="27" builtinId="34"/>
+    <cellStyle name="标题 4" xfId="28" builtinId="19"/>
+    <cellStyle name="货币[0]" xfId="29" builtinId="7"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="30" builtinId="43"/>
+    <cellStyle name="千位分隔" xfId="31" builtinId="3"/>
+    <cellStyle name="已访问的超链接" xfId="32" builtinId="9"/>
+    <cellStyle name="标题" xfId="33" builtinId="15"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="34" builtinId="35"/>
+    <cellStyle name="警告文本" xfId="35" builtinId="11"/>
     <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+    <cellStyle name="注释" xfId="37" builtinId="10"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="38" builtinId="50"/>
+    <cellStyle name="强调文字颜色 5" xfId="39" builtinId="45"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="40" builtinId="51"/>
+    <cellStyle name="超链接" xfId="41" builtinId="8"/>
+    <cellStyle name="千位分隔[0]" xfId="42" builtinId="6"/>
+    <cellStyle name="标题 2" xfId="43" builtinId="17"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
+    <cellStyle name="标题 3" xfId="45" builtinId="18"/>
+    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="47" builtinId="31"/>
+    <cellStyle name="链接单元格" xfId="48" builtinId="24"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -2332,8 +1956,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4664075" y="12668250"/>
-          <a:ext cx="4214495" cy="4984750"/>
+          <a:off x="4622800" y="12668250"/>
+          <a:ext cx="4171315" cy="4984750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2368,8 +1992,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4162425" y="635000"/>
-          <a:ext cx="4243070" cy="4984750"/>
+          <a:off x="4123690" y="635000"/>
+          <a:ext cx="4203065" cy="4984750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2416,8 +2040,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm rot="5400000">
-          <a:off x="650240" y="-344170"/>
-          <a:ext cx="2829560" cy="3551555"/>
+          <a:off x="368935" y="-62230"/>
+          <a:ext cx="3358515" cy="3517265"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2692,7 +2316,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:H129"/>
-  <sheetFormatPr defaultColWidth="14" defaultRowHeight="12.75" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="14" defaultRowHeight="15.2" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -3699,7 +3323,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C673"/>
-  <sheetFormatPr defaultColWidth="14" defaultRowHeight="12.75" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="14" defaultRowHeight="15.2" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
@@ -3823,81 +3447,51 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:3">
-      <c r="A12" s="14" t="s">
-        <v>263</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>264</v>
-      </c>
-      <c r="C12" s="14">
-        <v>1</v>
-      </c>
+      <c r="A12" s="14"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:3">
       <c r="A13" s="14" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C13" s="14">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:3">
       <c r="A14" s="14" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C14" s="14">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:3">
-      <c r="A15" s="14" t="s">
-        <v>269</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>270</v>
-      </c>
-      <c r="C15" s="14">
-        <v>1</v>
-      </c>
+      <c r="A15" s="14"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="14"/>
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:3">
-      <c r="A16" s="14" t="s">
-        <v>271</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>272</v>
-      </c>
-      <c r="C16" s="14">
-        <v>1</v>
-      </c>
+      <c r="A16" s="14"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:3">
-      <c r="A17" s="14" t="s">
-        <v>273</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>274</v>
-      </c>
-      <c r="C17" s="14">
-        <v>1</v>
-      </c>
+      <c r="A17" s="14"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:3">
-      <c r="A18" s="14" t="s">
-        <v>275</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>276</v>
-      </c>
-      <c r="C18" s="14">
-        <v>1</v>
-      </c>
+      <c r="A18" s="14"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:3">
       <c r="A19" s="14"/>
@@ -3906,224 +3500,104 @@
     </row>
     <row r="20" ht="15" customHeight="1"/>
     <row r="21" ht="15" customHeight="1" spans="1:3">
-      <c r="A21" s="14" t="s">
-        <v>277</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>278</v>
-      </c>
-      <c r="C21" s="14">
-        <v>2</v>
-      </c>
+      <c r="A21" s="14"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:3">
-      <c r="A22" s="14" t="s">
-        <v>279</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>280</v>
-      </c>
-      <c r="C22" s="14">
-        <v>2</v>
-      </c>
+      <c r="A22" s="14"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="14"/>
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:3">
-      <c r="A23" s="14" t="s">
-        <v>281</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>282</v>
-      </c>
-      <c r="C23" s="14">
-        <v>2</v>
-      </c>
+      <c r="A23" s="14"/>
+      <c r="B23" s="14"/>
+      <c r="C23" s="14"/>
     </row>
     <row r="24" ht="15" customHeight="1" spans="1:3">
-      <c r="A24" s="14" t="s">
-        <v>283</v>
-      </c>
-      <c r="B24" s="14" t="s">
-        <v>284</v>
-      </c>
-      <c r="C24" s="14">
-        <v>2</v>
-      </c>
+      <c r="A24" s="14"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
     </row>
     <row r="25" ht="15" customHeight="1" spans="1:3">
-      <c r="A25" s="14" t="s">
-        <v>285</v>
-      </c>
-      <c r="B25" s="14" t="s">
-        <v>286</v>
-      </c>
-      <c r="C25" s="14">
-        <v>2</v>
-      </c>
+      <c r="A25" s="14"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="14"/>
     </row>
     <row r="26" ht="15" customHeight="1" spans="1:3">
-      <c r="A26" s="14" t="s">
-        <v>287</v>
-      </c>
-      <c r="B26" s="14" t="s">
-        <v>288</v>
-      </c>
-      <c r="C26" s="14">
-        <v>2</v>
-      </c>
+      <c r="A26" s="14"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
     </row>
     <row r="27" ht="15" customHeight="1" spans="1:3">
-      <c r="A27" s="14" t="s">
-        <v>289</v>
-      </c>
-      <c r="B27" s="14" t="s">
-        <v>290</v>
-      </c>
-      <c r="C27" s="14">
-        <v>2</v>
-      </c>
+      <c r="A27" s="14"/>
+      <c r="B27" s="14"/>
+      <c r="C27" s="14"/>
     </row>
     <row r="28" ht="15" customHeight="1" spans="1:3">
-      <c r="A28" s="14" t="s">
-        <v>291</v>
-      </c>
-      <c r="B28" s="14" t="s">
-        <v>292</v>
-      </c>
-      <c r="C28" s="14">
-        <v>2</v>
-      </c>
+      <c r="A28" s="14"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
     </row>
     <row r="29" ht="15" customHeight="1" spans="1:3">
-      <c r="A29" s="14" t="s">
-        <v>293</v>
-      </c>
-      <c r="B29" s="14" t="s">
-        <v>294</v>
-      </c>
-      <c r="C29" s="14">
-        <v>2</v>
-      </c>
+      <c r="A29" s="14"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="14"/>
     </row>
     <row r="30" ht="15" customHeight="1" spans="1:3">
-      <c r="A30" s="14" t="s">
-        <v>295</v>
-      </c>
-      <c r="B30" s="14" t="s">
-        <v>296</v>
-      </c>
-      <c r="C30" s="14">
-        <v>2</v>
-      </c>
+      <c r="A30" s="14"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
     </row>
     <row r="31" ht="15" customHeight="1" spans="1:3">
-      <c r="A31" s="14" t="s">
-        <v>297</v>
-      </c>
-      <c r="B31" s="14" t="s">
-        <v>298</v>
-      </c>
-      <c r="C31" s="14">
-        <v>2</v>
-      </c>
+      <c r="A31" s="14"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="14"/>
     </row>
     <row r="32" ht="15" customHeight="1" spans="1:3">
-      <c r="A32" s="14" t="s">
-        <v>299</v>
-      </c>
-      <c r="B32" s="14" t="s">
-        <v>300</v>
-      </c>
-      <c r="C32" s="14">
-        <v>2</v>
-      </c>
+      <c r="A32" s="14"/>
+      <c r="B32" s="14"/>
+      <c r="C32" s="14"/>
     </row>
     <row r="33" ht="15" customHeight="1" spans="1:3">
-      <c r="A33" s="14" t="s">
-        <v>301</v>
-      </c>
-      <c r="B33" s="14" t="s">
-        <v>302</v>
-      </c>
-      <c r="C33" s="14">
-        <v>2</v>
-      </c>
+      <c r="A33" s="14"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
     </row>
     <row r="34" ht="15" customHeight="1" spans="1:3">
-      <c r="A34" s="14" t="s">
-        <v>303</v>
-      </c>
-      <c r="B34" s="14" t="s">
-        <v>304</v>
-      </c>
-      <c r="C34" s="14">
-        <v>2</v>
-      </c>
+      <c r="A34" s="14"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="14"/>
     </row>
     <row r="35" ht="15" customHeight="1" spans="1:3">
-      <c r="A35" s="14" t="s">
-        <v>305</v>
-      </c>
-      <c r="B35" s="14" t="s">
-        <v>306</v>
-      </c>
-      <c r="C35" s="14">
-        <v>2</v>
-      </c>
+      <c r="A35" s="14"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="14"/>
     </row>
     <row r="36" ht="15" customHeight="1" spans="1:3">
-      <c r="A36" s="14" t="s">
-        <v>307</v>
-      </c>
-      <c r="B36" s="14" t="s">
-        <v>308</v>
-      </c>
-      <c r="C36" s="14">
-        <v>2</v>
-      </c>
+      <c r="A36" s="14"/>
+      <c r="B36" s="14"/>
+      <c r="C36" s="14"/>
     </row>
     <row r="37" ht="15" customHeight="1" spans="1:3">
-      <c r="A37" s="14" t="s">
-        <v>309</v>
-      </c>
-      <c r="B37" s="14" t="s">
-        <v>310</v>
-      </c>
-      <c r="C37" s="14">
-        <v>2</v>
-      </c>
+      <c r="A37" s="14"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="14"/>
     </row>
     <row r="38" ht="15" customHeight="1" spans="1:3">
-      <c r="A38" s="14" t="s">
-        <v>311</v>
-      </c>
-      <c r="B38" s="14" t="s">
-        <v>312</v>
-      </c>
-      <c r="C38" s="14">
-        <v>2</v>
-      </c>
+      <c r="A38" s="14"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="14"/>
     </row>
     <row r="39" ht="15" customHeight="1" spans="1:3">
-      <c r="A39" s="14" t="s">
-        <v>313</v>
-      </c>
-      <c r="B39" s="14" t="s">
-        <v>314</v>
-      </c>
-      <c r="C39" s="14">
-        <v>2</v>
-      </c>
+      <c r="A39" s="14"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="14"/>
     </row>
     <row r="40" ht="15" customHeight="1" spans="1:3">
-      <c r="A40" s="14" t="s">
-        <v>315</v>
-      </c>
-      <c r="B40" s="14" t="s">
-        <v>316</v>
-      </c>
-      <c r="C40" s="14">
-        <v>2</v>
-      </c>
+      <c r="A40" s="14"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="14"/>
     </row>
     <row r="41" ht="15" customHeight="1" spans="1:3">
       <c r="A41" s="14"/>
@@ -4141,357 +3615,165 @@
       <c r="C43" s="14"/>
     </row>
     <row r="44" ht="15" customHeight="1" spans="1:3">
-      <c r="A44" s="12" t="s">
-        <v>317</v>
-      </c>
-      <c r="B44" s="12" t="s">
-        <v>318</v>
-      </c>
-      <c r="C44" s="12">
-        <v>3</v>
-      </c>
+      <c r="A44" s="12"/>
+      <c r="B44" s="12"/>
+      <c r="C44" s="12"/>
     </row>
     <row r="45" ht="15" customHeight="1" spans="1:3">
-      <c r="A45" s="12" t="s">
-        <v>319</v>
-      </c>
-      <c r="B45" s="12" t="s">
-        <v>320</v>
-      </c>
-      <c r="C45" s="12">
-        <v>3</v>
-      </c>
+      <c r="A45" s="12"/>
+      <c r="B45" s="12"/>
+      <c r="C45" s="12"/>
     </row>
     <row r="46" ht="15" customHeight="1" spans="1:3">
-      <c r="A46" s="12" t="s">
-        <v>321</v>
-      </c>
-      <c r="B46" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="C46" s="12">
-        <v>3</v>
-      </c>
+      <c r="A46" s="12"/>
+      <c r="B46" s="12"/>
+      <c r="C46" s="12"/>
     </row>
     <row r="47" ht="15" customHeight="1" spans="1:3">
-      <c r="A47" s="12" t="s">
-        <v>323</v>
-      </c>
-      <c r="B47" s="12" t="s">
-        <v>324</v>
-      </c>
-      <c r="C47" s="12">
-        <v>3</v>
-      </c>
+      <c r="A47" s="12"/>
+      <c r="B47" s="12"/>
+      <c r="C47" s="12"/>
     </row>
     <row r="48" ht="15" customHeight="1" spans="1:3">
-      <c r="A48" s="12" t="s">
-        <v>325</v>
-      </c>
-      <c r="B48" s="12" t="s">
-        <v>326</v>
-      </c>
-      <c r="C48" s="12">
-        <v>3</v>
-      </c>
+      <c r="A48" s="12"/>
+      <c r="B48" s="12"/>
+      <c r="C48" s="12"/>
     </row>
     <row r="49" ht="15" customHeight="1" spans="1:3">
-      <c r="A49" s="12" t="s">
-        <v>327</v>
-      </c>
-      <c r="B49" s="12" t="s">
-        <v>328</v>
-      </c>
-      <c r="C49" s="12">
-        <v>3</v>
-      </c>
+      <c r="A49" s="12"/>
+      <c r="B49" s="12"/>
+      <c r="C49" s="12"/>
     </row>
     <row r="50" ht="15" customHeight="1" spans="1:3">
-      <c r="A50" s="12" t="s">
-        <v>329</v>
-      </c>
-      <c r="B50" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="C50" s="12">
-        <v>3</v>
-      </c>
+      <c r="A50" s="12"/>
+      <c r="B50" s="12"/>
+      <c r="C50" s="12"/>
     </row>
     <row r="51" ht="15" customHeight="1" spans="1:3">
-      <c r="A51" s="12" t="s">
-        <v>331</v>
-      </c>
-      <c r="B51" s="12" t="s">
-        <v>332</v>
-      </c>
-      <c r="C51" s="12">
-        <v>3</v>
-      </c>
+      <c r="A51" s="12"/>
+      <c r="B51" s="12"/>
+      <c r="C51" s="12"/>
     </row>
     <row r="52" ht="15" customHeight="1" spans="1:3">
-      <c r="A52" s="12" t="s">
-        <v>333</v>
-      </c>
-      <c r="B52" s="12" t="s">
-        <v>334</v>
-      </c>
-      <c r="C52" s="12">
-        <v>3</v>
-      </c>
+      <c r="A52" s="12"/>
+      <c r="B52" s="12"/>
+      <c r="C52" s="12"/>
     </row>
     <row r="53" ht="15" customHeight="1" spans="1:3">
-      <c r="A53" s="12" t="s">
-        <v>335</v>
-      </c>
-      <c r="B53" s="12" t="s">
-        <v>336</v>
-      </c>
-      <c r="C53" s="12">
-        <v>3</v>
-      </c>
+      <c r="A53" s="12"/>
+      <c r="B53" s="12"/>
+      <c r="C53" s="12"/>
     </row>
     <row r="54" ht="15" customHeight="1" spans="1:3">
-      <c r="A54" s="12" t="s">
-        <v>337</v>
-      </c>
-      <c r="B54" s="12" t="s">
-        <v>338</v>
-      </c>
-      <c r="C54" s="12">
-        <v>3</v>
-      </c>
+      <c r="A54" s="12"/>
+      <c r="B54" s="12"/>
+      <c r="C54" s="12"/>
     </row>
     <row r="55" ht="15" customHeight="1" spans="1:3">
-      <c r="A55" s="12" t="s">
-        <v>339</v>
-      </c>
-      <c r="B55" s="12" t="s">
-        <v>340</v>
-      </c>
-      <c r="C55" s="12">
-        <v>3</v>
-      </c>
+      <c r="A55" s="12"/>
+      <c r="B55" s="12"/>
+      <c r="C55" s="12"/>
     </row>
     <row r="56" ht="15" customHeight="1"/>
     <row r="57" ht="15" customHeight="1" spans="1:3">
-      <c r="A57" s="12" t="s">
-        <v>341</v>
-      </c>
-      <c r="B57" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="C57" s="12">
-        <v>4</v>
-      </c>
+      <c r="A57" s="12"/>
+      <c r="B57" s="12"/>
+      <c r="C57" s="12"/>
     </row>
     <row r="58" ht="15" customHeight="1" spans="1:3">
-      <c r="A58" s="12" t="s">
-        <v>343</v>
-      </c>
-      <c r="B58" s="12" t="s">
-        <v>344</v>
-      </c>
-      <c r="C58" s="12">
-        <v>4</v>
-      </c>
+      <c r="A58" s="12"/>
+      <c r="B58" s="12"/>
+      <c r="C58" s="12"/>
     </row>
     <row r="59" ht="15" customHeight="1" spans="1:3">
-      <c r="A59" s="12" t="s">
-        <v>345</v>
-      </c>
-      <c r="B59" s="12" t="s">
-        <v>346</v>
-      </c>
-      <c r="C59" s="12">
-        <v>4</v>
-      </c>
+      <c r="A59" s="12"/>
+      <c r="B59" s="12"/>
+      <c r="C59" s="12"/>
     </row>
     <row r="60" ht="15" customHeight="1" spans="1:3">
-      <c r="A60" s="12" t="s">
-        <v>347</v>
-      </c>
-      <c r="B60" s="12" t="s">
-        <v>348</v>
-      </c>
-      <c r="C60" s="12">
-        <v>4</v>
-      </c>
+      <c r="A60" s="12"/>
+      <c r="B60" s="12"/>
+      <c r="C60" s="12"/>
     </row>
     <row r="61" ht="15" customHeight="1" spans="1:3">
-      <c r="A61" s="12" t="s">
-        <v>349</v>
-      </c>
-      <c r="B61" s="12" t="s">
-        <v>350</v>
-      </c>
-      <c r="C61" s="12">
-        <v>4</v>
-      </c>
+      <c r="A61" s="12"/>
+      <c r="B61" s="12"/>
+      <c r="C61" s="12"/>
     </row>
     <row r="62" ht="15" customHeight="1" spans="1:3">
-      <c r="A62" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="B62" s="12" t="s">
-        <v>352</v>
-      </c>
-      <c r="C62" s="12">
-        <v>4</v>
-      </c>
+      <c r="A62" s="12"/>
+      <c r="B62" s="12"/>
+      <c r="C62" s="12"/>
     </row>
     <row r="63" ht="15" customHeight="1" spans="1:3">
-      <c r="A63" s="12" t="s">
-        <v>353</v>
-      </c>
-      <c r="B63" s="12" t="s">
-        <v>354</v>
-      </c>
-      <c r="C63" s="12">
-        <v>4</v>
-      </c>
+      <c r="A63" s="12"/>
+      <c r="B63" s="12"/>
+      <c r="C63" s="12"/>
     </row>
     <row r="64" ht="15" customHeight="1" spans="1:3">
-      <c r="A64" s="12" t="s">
-        <v>355</v>
-      </c>
-      <c r="B64" s="12" t="s">
-        <v>356</v>
-      </c>
-      <c r="C64" s="12">
-        <v>4</v>
-      </c>
+      <c r="A64" s="12"/>
+      <c r="B64" s="12"/>
+      <c r="C64" s="12"/>
     </row>
     <row r="65" ht="15" customHeight="1" spans="1:3">
-      <c r="A65" s="12" t="s">
-        <v>357</v>
-      </c>
-      <c r="B65" s="12" t="s">
-        <v>358</v>
-      </c>
-      <c r="C65" s="12">
-        <v>4</v>
-      </c>
+      <c r="A65" s="12"/>
+      <c r="B65" s="12"/>
+      <c r="C65" s="12"/>
     </row>
     <row r="66" ht="15" customHeight="1" spans="1:3">
-      <c r="A66" s="12" t="s">
-        <v>359</v>
-      </c>
-      <c r="B66" s="12" t="s">
-        <v>360</v>
-      </c>
-      <c r="C66" s="12">
-        <v>4</v>
-      </c>
+      <c r="A66" s="12"/>
+      <c r="B66" s="12"/>
+      <c r="C66" s="12"/>
     </row>
     <row r="67" ht="15" customHeight="1" spans="1:3">
-      <c r="A67" s="12" t="s">
-        <v>361</v>
-      </c>
-      <c r="B67" s="12" t="s">
-        <v>362</v>
-      </c>
-      <c r="C67" s="12">
-        <v>4</v>
-      </c>
+      <c r="A67" s="12"/>
+      <c r="B67" s="12"/>
+      <c r="C67" s="12"/>
     </row>
     <row r="68" ht="15" customHeight="1" spans="1:3">
-      <c r="A68" s="12" t="s">
-        <v>363</v>
-      </c>
-      <c r="B68" s="12" t="s">
-        <v>364</v>
-      </c>
-      <c r="C68" s="12">
-        <v>4</v>
-      </c>
+      <c r="A68" s="12"/>
+      <c r="B68" s="12"/>
+      <c r="C68" s="12"/>
     </row>
     <row r="69" ht="15" customHeight="1" spans="1:3">
-      <c r="A69" s="12" t="s">
-        <v>365</v>
-      </c>
-      <c r="B69" s="12" t="s">
-        <v>366</v>
-      </c>
-      <c r="C69" s="12">
-        <v>4</v>
-      </c>
+      <c r="A69" s="12"/>
+      <c r="B69" s="12"/>
+      <c r="C69" s="12"/>
     </row>
     <row r="70" ht="15" customHeight="1" spans="1:3">
-      <c r="A70" s="12" t="s">
-        <v>367</v>
-      </c>
-      <c r="B70" s="12" t="s">
-        <v>368</v>
-      </c>
-      <c r="C70" s="12">
-        <v>4</v>
-      </c>
+      <c r="A70" s="12"/>
+      <c r="B70" s="12"/>
+      <c r="C70" s="12"/>
     </row>
     <row r="71" ht="15" customHeight="1" spans="1:3">
-      <c r="A71" s="12" t="s">
-        <v>369</v>
-      </c>
-      <c r="B71" s="12" t="s">
-        <v>370</v>
-      </c>
-      <c r="C71" s="12">
-        <v>4</v>
-      </c>
+      <c r="A71" s="12"/>
+      <c r="B71" s="12"/>
+      <c r="C71" s="12"/>
     </row>
     <row r="72" ht="15" customHeight="1" spans="1:3">
-      <c r="A72" s="12" t="s">
-        <v>371</v>
-      </c>
-      <c r="B72" s="12" t="s">
-        <v>372</v>
-      </c>
-      <c r="C72" s="12">
-        <v>4</v>
-      </c>
+      <c r="A72" s="12"/>
+      <c r="B72" s="12"/>
+      <c r="C72" s="12"/>
     </row>
     <row r="73" ht="15" customHeight="1" spans="1:3">
-      <c r="A73" s="12" t="s">
-        <v>373</v>
-      </c>
-      <c r="B73" s="12" t="s">
-        <v>374</v>
-      </c>
-      <c r="C73" s="12">
-        <v>4</v>
-      </c>
+      <c r="A73" s="12"/>
+      <c r="B73" s="12"/>
+      <c r="C73" s="12"/>
     </row>
     <row r="74" ht="15" customHeight="1" spans="1:3">
-      <c r="A74" s="12" t="s">
-        <v>375</v>
-      </c>
-      <c r="B74" s="12" t="s">
-        <v>376</v>
-      </c>
-      <c r="C74" s="12">
-        <v>4</v>
-      </c>
+      <c r="A74" s="12"/>
+      <c r="B74" s="12"/>
+      <c r="C74" s="12"/>
     </row>
     <row r="75" ht="15" customHeight="1" spans="1:3">
-      <c r="A75" s="12" t="s">
-        <v>377</v>
-      </c>
-      <c r="B75" s="12" t="s">
-        <v>378</v>
-      </c>
-      <c r="C75" s="12">
-        <v>4</v>
-      </c>
+      <c r="A75" s="12"/>
+      <c r="B75" s="12"/>
+      <c r="C75" s="12"/>
     </row>
     <row r="76" ht="15" customHeight="1" spans="1:3">
-      <c r="A76" s="12" t="s">
-        <v>379</v>
-      </c>
-      <c r="B76" s="12" t="s">
-        <v>380</v>
-      </c>
-      <c r="C76" s="12">
-        <v>4</v>
-      </c>
+      <c r="A76" s="12"/>
+      <c r="B76" s="12"/>
+      <c r="C76" s="12"/>
     </row>
     <row r="77" ht="15" customHeight="1" spans="1:3">
       <c r="A77" s="14"/>
@@ -7409,7 +6691,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C90"/>
-  <sheetFormatPr defaultColWidth="14" defaultRowHeight="12.75" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="14" defaultRowHeight="15.2" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="37" customWidth="1"/>
     <col min="2" max="20" width="9" customWidth="1"/>
@@ -7420,7 +6702,7 @@
         <v>245</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>381</v>
+        <v>267</v>
       </c>
       <c r="C1" s="11">
         <v>0</v>
@@ -7431,7 +6713,7 @@
         <v>247</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>381</v>
+        <v>267</v>
       </c>
       <c r="C2" s="11">
         <v>1</v>
@@ -7442,7 +6724,7 @@
         <v>249</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>381</v>
+        <v>267</v>
       </c>
       <c r="C3" s="11">
         <v>2</v>
@@ -7453,7 +6735,7 @@
         <v>252</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>381</v>
+        <v>267</v>
       </c>
       <c r="C4" s="11">
         <v>3</v>
@@ -7461,10 +6743,10 @@
     </row>
     <row r="5" ht="15" customHeight="1" spans="1:3">
       <c r="A5" s="12" t="s">
-        <v>382</v>
+        <v>268</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>381</v>
+        <v>267</v>
       </c>
       <c r="C5" s="11">
         <v>4</v>
@@ -7472,10 +6754,10 @@
     </row>
     <row r="6" ht="15" customHeight="1" spans="1:3">
       <c r="A6" s="12" t="s">
-        <v>383</v>
+        <v>269</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>381</v>
+        <v>267</v>
       </c>
       <c r="C6" s="11">
         <v>5</v>
@@ -7483,10 +6765,10 @@
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:3">
       <c r="A7" s="12" t="s">
-        <v>384</v>
+        <v>270</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>381</v>
+        <v>267</v>
       </c>
       <c r="C7" s="11">
         <v>6</v>
@@ -7494,10 +6776,10 @@
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:3">
       <c r="A8" s="12" t="s">
-        <v>385</v>
+        <v>271</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>381</v>
+        <v>267</v>
       </c>
       <c r="C8" s="11">
         <v>7</v>
@@ -7505,10 +6787,10 @@
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:3">
       <c r="A9" s="12" t="s">
-        <v>386</v>
+        <v>253</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>381</v>
+        <v>267</v>
       </c>
       <c r="C9" s="11">
         <v>8</v>
@@ -7516,10 +6798,10 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:3">
       <c r="A10" s="12" t="s">
-        <v>387</v>
+        <v>255</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>381</v>
+        <v>267</v>
       </c>
       <c r="C10" s="11">
         <v>9</v>
@@ -7527,10 +6809,10 @@
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:3">
       <c r="A11" s="12" t="s">
-        <v>388</v>
+        <v>257</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>381</v>
+        <v>267</v>
       </c>
       <c r="C11" s="11">
         <v>10</v>
@@ -7538,10 +6820,10 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:3">
       <c r="A12" s="12" t="s">
-        <v>389</v>
+        <v>259</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>381</v>
+        <v>267</v>
       </c>
       <c r="C12" s="11">
         <v>11</v>
@@ -7549,10 +6831,10 @@
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:3">
       <c r="A13" s="12" t="s">
-        <v>390</v>
+        <v>263</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>381</v>
+        <v>267</v>
       </c>
       <c r="C13" s="11">
         <v>12</v>
@@ -7560,10 +6842,10 @@
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:3">
       <c r="A14" s="12" t="s">
-        <v>391</v>
+        <v>262</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>381</v>
+        <v>267</v>
       </c>
       <c r="C14" s="11">
         <v>13</v>
@@ -7571,10 +6853,10 @@
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:3">
       <c r="A15" s="12" t="s">
-        <v>392</v>
+        <v>266</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>381</v>
+        <v>267</v>
       </c>
       <c r="C15" s="11">
         <v>14</v>
@@ -7587,10 +6869,10 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:3">
       <c r="A17" s="10" t="s">
-        <v>393</v>
+        <v>272</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>394</v>
+        <v>273</v>
       </c>
       <c r="C17" s="13">
         <v>15</v>
@@ -7598,10 +6880,10 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:3">
       <c r="A18" s="10" t="s">
-        <v>395</v>
+        <v>274</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>394</v>
+        <v>273</v>
       </c>
       <c r="C18" s="13">
         <v>14</v>
@@ -7609,10 +6891,10 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:3">
       <c r="A19" s="10" t="s">
-        <v>396</v>
+        <v>275</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>394</v>
+        <v>273</v>
       </c>
       <c r="C19" s="13">
         <v>13</v>
@@ -7620,103 +6902,103 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:3">
       <c r="A20" s="10" t="s">
-        <v>397</v>
+        <v>276</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>394</v>
+        <v>273</v>
       </c>
       <c r="C20" s="13">
         <v>12</v>
       </c>
     </row>
-    <row r="21" ht="13.85" spans="1:3">
+    <row r="21" ht="16.8" spans="1:3">
       <c r="A21" s="12"/>
       <c r="B21" s="11"/>
       <c r="C21" s="11"/>
     </row>
-    <row r="22" ht="13.85" spans="1:3">
+    <row r="22" ht="16.8" spans="1:3">
       <c r="A22" s="10" t="s">
-        <v>398</v>
+        <v>277</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>399</v>
+        <v>278</v>
       </c>
       <c r="C22" s="13">
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="13.85" spans="1:3">
+    <row r="23" ht="16.8" spans="1:3">
       <c r="A23" s="10" t="s">
-        <v>400</v>
+        <v>279</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>399</v>
+        <v>278</v>
       </c>
       <c r="C23" s="13">
         <v>1</v>
       </c>
     </row>
-    <row r="24" ht="13.85" spans="1:3">
+    <row r="24" ht="16.8" spans="1:3">
       <c r="A24" s="10" t="s">
-        <v>401</v>
+        <v>280</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>399</v>
+        <v>278</v>
       </c>
       <c r="C24" s="13">
         <v>2</v>
       </c>
     </row>
-    <row r="25" ht="13.85" spans="1:3">
+    <row r="25" ht="16.8" spans="1:3">
       <c r="A25" s="10" t="s">
-        <v>402</v>
+        <v>281</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>399</v>
+        <v>278</v>
       </c>
       <c r="C25" s="13">
         <v>3</v>
       </c>
     </row>
-    <row r="26" ht="13.85" spans="1:3">
+    <row r="26" ht="16.8" spans="1:3">
       <c r="A26" s="10" t="s">
-        <v>403</v>
+        <v>282</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>399</v>
+        <v>278</v>
       </c>
       <c r="C26" s="13">
         <v>4</v>
       </c>
     </row>
-    <row r="27" ht="13.85" spans="1:3">
+    <row r="27" ht="16.8" spans="1:3">
       <c r="A27" s="10" t="s">
-        <v>404</v>
+        <v>283</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>399</v>
+        <v>278</v>
       </c>
       <c r="C27" s="13">
         <v>5</v>
       </c>
     </row>
-    <row r="28" ht="13.85" spans="1:3">
+    <row r="28" ht="16.8" spans="1:3">
       <c r="A28" s="10" t="s">
-        <v>405</v>
+        <v>284</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>399</v>
+        <v>278</v>
       </c>
       <c r="C28" s="13">
         <v>6</v>
       </c>
     </row>
-    <row r="29" ht="13.85" spans="1:3">
+    <row r="29" ht="16.8" spans="1:3">
       <c r="A29" s="10" t="s">
-        <v>406</v>
+        <v>285</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>399</v>
+        <v>278</v>
       </c>
       <c r="C29" s="13">
         <v>7</v>
@@ -7727,89 +7009,89 @@
       <c r="B30" s="13"/>
       <c r="C30" s="13"/>
     </row>
-    <row r="31" ht="13.85" spans="1:3">
+    <row r="31" ht="16.8" spans="1:3">
       <c r="A31" s="10" t="s">
-        <v>407</v>
+        <v>286</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>408</v>
+        <v>287</v>
       </c>
       <c r="C31" s="13">
         <v>0</v>
       </c>
     </row>
-    <row r="32" ht="13.85" spans="1:3">
+    <row r="32" ht="16.8" spans="1:3">
       <c r="A32" s="10" t="s">
-        <v>409</v>
+        <v>288</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>408</v>
+        <v>287</v>
       </c>
       <c r="C32" s="13">
         <v>1</v>
       </c>
     </row>
-    <row r="33" ht="13.85" spans="1:3">
+    <row r="33" ht="16.8" spans="1:3">
       <c r="A33" s="10" t="s">
-        <v>410</v>
+        <v>289</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>408</v>
+        <v>287</v>
       </c>
       <c r="C33" s="13">
         <v>2</v>
       </c>
     </row>
-    <row r="34" ht="13.85" spans="1:3">
+    <row r="34" ht="16.8" spans="1:3">
       <c r="A34" s="10" t="s">
-        <v>411</v>
+        <v>290</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>408</v>
+        <v>287</v>
       </c>
       <c r="C34" s="13">
         <v>3</v>
       </c>
     </row>
-    <row r="35" ht="13.85" spans="1:3">
+    <row r="35" ht="16.8" spans="1:3">
       <c r="A35" s="10" t="s">
-        <v>412</v>
+        <v>291</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>408</v>
+        <v>287</v>
       </c>
       <c r="C35" s="13">
         <v>4</v>
       </c>
     </row>
-    <row r="36" ht="13.85" spans="1:3">
+    <row r="36" ht="16.8" spans="1:3">
       <c r="A36" s="10" t="s">
-        <v>413</v>
+        <v>292</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>408</v>
+        <v>287</v>
       </c>
       <c r="C36" s="13">
         <v>5</v>
       </c>
     </row>
-    <row r="37" ht="13.85" spans="1:3">
+    <row r="37" ht="16.8" spans="1:3">
       <c r="A37" s="10" t="s">
-        <v>414</v>
+        <v>293</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>408</v>
+        <v>287</v>
       </c>
       <c r="C37" s="13">
         <v>6</v>
       </c>
     </row>
-    <row r="38" ht="13.85" spans="1:3">
+    <row r="38" ht="16.8" spans="1:3">
       <c r="A38" s="10" t="s">
-        <v>415</v>
+        <v>294</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>408</v>
+        <v>287</v>
       </c>
       <c r="C38" s="13">
         <v>7</v>
@@ -7820,89 +7102,89 @@
       <c r="B39" s="13"/>
       <c r="C39" s="13"/>
     </row>
-    <row r="40" ht="13.85" spans="1:3">
+    <row r="40" ht="16.8" spans="1:3">
       <c r="A40" s="10" t="s">
-        <v>416</v>
+        <v>295</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>417</v>
+        <v>296</v>
       </c>
       <c r="C40" s="13">
         <v>0</v>
       </c>
     </row>
-    <row r="41" ht="13.85" spans="1:3">
+    <row r="41" ht="16.8" spans="1:3">
       <c r="A41" s="10" t="s">
-        <v>418</v>
+        <v>297</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>417</v>
+        <v>296</v>
       </c>
       <c r="C41" s="13">
         <v>1</v>
       </c>
     </row>
-    <row r="42" ht="13.85" spans="1:3">
+    <row r="42" ht="16.8" spans="1:3">
       <c r="A42" s="10" t="s">
-        <v>419</v>
+        <v>298</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>417</v>
+        <v>296</v>
       </c>
       <c r="C42" s="13">
         <v>2</v>
       </c>
     </row>
-    <row r="43" ht="13.85" spans="1:3">
+    <row r="43" ht="16.8" spans="1:3">
       <c r="A43" s="10" t="s">
-        <v>420</v>
+        <v>299</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>417</v>
+        <v>296</v>
       </c>
       <c r="C43" s="13">
         <v>3</v>
       </c>
     </row>
-    <row r="44" ht="13.85" spans="1:3">
+    <row r="44" ht="16.8" spans="1:3">
       <c r="A44" s="10" t="s">
-        <v>421</v>
+        <v>300</v>
       </c>
       <c r="B44" s="13" t="s">
-        <v>417</v>
+        <v>296</v>
       </c>
       <c r="C44" s="13">
         <v>4</v>
       </c>
     </row>
-    <row r="45" ht="13.85" spans="1:3">
+    <row r="45" ht="16.8" spans="1:3">
       <c r="A45" s="10" t="s">
-        <v>422</v>
+        <v>301</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>417</v>
+        <v>296</v>
       </c>
       <c r="C45" s="13">
         <v>5</v>
       </c>
     </row>
-    <row r="46" ht="13.85" spans="1:3">
+    <row r="46" ht="16.8" spans="1:3">
       <c r="A46" s="10" t="s">
-        <v>423</v>
+        <v>302</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>417</v>
+        <v>296</v>
       </c>
       <c r="C46" s="13">
         <v>6</v>
       </c>
     </row>
-    <row r="47" ht="13.85" spans="1:3">
+    <row r="47" ht="16.8" spans="1:3">
       <c r="A47" s="10" t="s">
-        <v>424</v>
+        <v>303</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>417</v>
+        <v>296</v>
       </c>
       <c r="C47" s="13">
         <v>7</v>
@@ -7913,89 +7195,89 @@
       <c r="B48" s="13"/>
       <c r="C48" s="13"/>
     </row>
-    <row r="49" ht="13.85" spans="1:3">
+    <row r="49" ht="16.8" spans="1:3">
       <c r="A49" s="10" t="s">
-        <v>425</v>
+        <v>304</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>426</v>
+        <v>305</v>
       </c>
       <c r="C49" s="13">
         <v>0</v>
       </c>
     </row>
-    <row r="50" ht="13.85" spans="1:3">
+    <row r="50" ht="16.8" spans="1:3">
       <c r="A50" s="10" t="s">
-        <v>427</v>
+        <v>306</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>426</v>
+        <v>305</v>
       </c>
       <c r="C50" s="13">
         <v>1</v>
       </c>
     </row>
-    <row r="51" ht="13.85" spans="1:3">
+    <row r="51" ht="16.8" spans="1:3">
       <c r="A51" s="10" t="s">
-        <v>428</v>
+        <v>307</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>426</v>
+        <v>305</v>
       </c>
       <c r="C51" s="13">
         <v>2</v>
       </c>
     </row>
-    <row r="52" ht="13.85" spans="1:3">
+    <row r="52" ht="16.8" spans="1:3">
       <c r="A52" s="10" t="s">
-        <v>429</v>
+        <v>308</v>
       </c>
       <c r="B52" s="13" t="s">
-        <v>426</v>
+        <v>305</v>
       </c>
       <c r="C52" s="13">
         <v>3</v>
       </c>
     </row>
-    <row r="53" ht="13.85" spans="1:3">
+    <row r="53" ht="16.8" spans="1:3">
       <c r="A53" s="10" t="s">
-        <v>430</v>
+        <v>309</v>
       </c>
       <c r="B53" s="13" t="s">
-        <v>426</v>
+        <v>305</v>
       </c>
       <c r="C53" s="13">
         <v>4</v>
       </c>
     </row>
-    <row r="54" ht="13.85" spans="1:3">
+    <row r="54" ht="16.8" spans="1:3">
       <c r="A54" s="10" t="s">
-        <v>431</v>
+        <v>310</v>
       </c>
       <c r="B54" s="13" t="s">
-        <v>426</v>
+        <v>305</v>
       </c>
       <c r="C54" s="13">
         <v>5</v>
       </c>
     </row>
-    <row r="55" ht="13.85" spans="1:3">
+    <row r="55" ht="16.8" spans="1:3">
       <c r="A55" s="10" t="s">
-        <v>432</v>
+        <v>311</v>
       </c>
       <c r="B55" s="13" t="s">
-        <v>426</v>
+        <v>305</v>
       </c>
       <c r="C55" s="13">
         <v>6</v>
       </c>
     </row>
-    <row r="56" ht="13.85" spans="1:3">
+    <row r="56" ht="16.8" spans="1:3">
       <c r="A56" s="10" t="s">
-        <v>433</v>
+        <v>312</v>
       </c>
       <c r="B56" s="13" t="s">
-        <v>426</v>
+        <v>305</v>
       </c>
       <c r="C56" s="13">
         <v>7</v>
@@ -8006,177 +7288,177 @@
       <c r="B57" s="11"/>
       <c r="C57" s="11"/>
     </row>
-    <row r="58" ht="13.85" spans="1:3">
+    <row r="58" ht="16.8" spans="1:3">
       <c r="A58" s="12" t="s">
-        <v>434</v>
+        <v>313</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>435</v>
+        <v>314</v>
       </c>
       <c r="C58" s="11">
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="13.85" spans="1:3">
+    <row r="59" ht="16.8" spans="1:3">
       <c r="A59" s="12" t="s">
-        <v>436</v>
+        <v>315</v>
       </c>
       <c r="B59" s="11" t="s">
-        <v>435</v>
+        <v>314</v>
       </c>
       <c r="C59" s="11">
         <v>1</v>
       </c>
     </row>
-    <row r="60" ht="13.85" spans="1:3">
+    <row r="60" ht="16.8" spans="1:3">
       <c r="A60" s="12" t="s">
-        <v>437</v>
+        <v>316</v>
       </c>
       <c r="B60" s="11" t="s">
-        <v>435</v>
+        <v>314</v>
       </c>
       <c r="C60" s="11">
         <v>2</v>
       </c>
     </row>
-    <row r="61" ht="13.85" spans="1:3">
+    <row r="61" ht="16.8" spans="1:3">
       <c r="A61" s="12" t="s">
-        <v>438</v>
+        <v>317</v>
       </c>
       <c r="B61" s="11" t="s">
-        <v>435</v>
+        <v>314</v>
       </c>
       <c r="C61" s="11">
         <v>3</v>
       </c>
     </row>
-    <row r="62" ht="13.85" spans="1:3">
+    <row r="62" ht="16.8" spans="1:3">
       <c r="A62" s="12" t="s">
-        <v>439</v>
+        <v>318</v>
       </c>
       <c r="B62" s="11" t="s">
-        <v>435</v>
+        <v>314</v>
       </c>
       <c r="C62" s="11">
         <v>4</v>
       </c>
     </row>
-    <row r="63" ht="13.85" spans="1:3">
+    <row r="63" ht="16.8" spans="1:3">
       <c r="A63" s="12" t="s">
-        <v>440</v>
+        <v>319</v>
       </c>
       <c r="B63" s="11" t="s">
-        <v>435</v>
+        <v>314</v>
       </c>
       <c r="C63" s="11">
         <v>5</v>
       </c>
     </row>
-    <row r="64" ht="13.85" spans="1:3">
+    <row r="64" ht="16.8" spans="1:3">
       <c r="A64" s="12" t="s">
-        <v>441</v>
+        <v>320</v>
       </c>
       <c r="B64" s="11" t="s">
-        <v>435</v>
+        <v>314</v>
       </c>
       <c r="C64" s="11">
         <v>6</v>
       </c>
     </row>
-    <row r="65" ht="13.85" spans="1:3">
+    <row r="65" ht="16.8" spans="1:3">
       <c r="A65" s="12" t="s">
-        <v>442</v>
+        <v>321</v>
       </c>
       <c r="B65" s="11" t="s">
-        <v>435</v>
+        <v>314</v>
       </c>
       <c r="C65" s="11">
         <v>7</v>
       </c>
     </row>
-    <row r="66" ht="13.85" spans="1:3">
+    <row r="66" ht="16.8" spans="1:3">
       <c r="A66" s="12" t="s">
-        <v>443</v>
+        <v>322</v>
       </c>
       <c r="B66" s="11" t="s">
-        <v>435</v>
+        <v>314</v>
       </c>
       <c r="C66" s="11">
         <v>8</v>
       </c>
     </row>
-    <row r="67" ht="13.85" spans="1:3">
+    <row r="67" ht="16.8" spans="1:3">
       <c r="A67" s="12" t="s">
-        <v>444</v>
+        <v>323</v>
       </c>
       <c r="B67" s="11" t="s">
-        <v>435</v>
+        <v>314</v>
       </c>
       <c r="C67" s="11">
         <v>9</v>
       </c>
     </row>
-    <row r="68" ht="13.85" spans="1:3">
+    <row r="68" ht="16.8" spans="1:3">
       <c r="A68" s="12" t="s">
-        <v>445</v>
+        <v>324</v>
       </c>
       <c r="B68" s="11" t="s">
-        <v>435</v>
+        <v>314</v>
       </c>
       <c r="C68" s="11">
         <v>10</v>
       </c>
     </row>
-    <row r="69" ht="13.85" spans="1:3">
+    <row r="69" ht="16.8" spans="1:3">
       <c r="A69" s="12" t="s">
-        <v>446</v>
+        <v>325</v>
       </c>
       <c r="B69" s="11" t="s">
-        <v>435</v>
+        <v>314</v>
       </c>
       <c r="C69" s="11">
         <v>11</v>
       </c>
     </row>
-    <row r="70" ht="13.85" spans="1:3">
+    <row r="70" ht="16.8" spans="1:3">
       <c r="A70" s="12" t="s">
-        <v>447</v>
+        <v>326</v>
       </c>
       <c r="B70" s="11" t="s">
-        <v>435</v>
+        <v>314</v>
       </c>
       <c r="C70" s="11">
         <v>12</v>
       </c>
     </row>
-    <row r="71" ht="13.85" spans="1:3">
+    <row r="71" ht="16.8" spans="1:3">
       <c r="A71" s="12" t="s">
-        <v>448</v>
+        <v>327</v>
       </c>
       <c r="B71" s="11" t="s">
-        <v>435</v>
+        <v>314</v>
       </c>
       <c r="C71" s="11">
         <v>13</v>
       </c>
     </row>
-    <row r="72" ht="13.85" spans="1:3">
+    <row r="72" ht="16.8" spans="1:3">
       <c r="A72" s="12" t="s">
-        <v>449</v>
+        <v>328</v>
       </c>
       <c r="B72" s="11" t="s">
-        <v>435</v>
+        <v>314</v>
       </c>
       <c r="C72" s="11">
         <v>14</v>
       </c>
     </row>
-    <row r="73" ht="13.85" spans="1:3">
+    <row r="73" ht="16.8" spans="1:3">
       <c r="A73" s="12" t="s">
-        <v>450</v>
+        <v>329</v>
       </c>
       <c r="B73" s="11" t="s">
-        <v>435</v>
+        <v>314</v>
       </c>
       <c r="C73" s="11">
         <v>15</v>
@@ -8187,177 +7469,177 @@
       <c r="B74" s="11"/>
       <c r="C74" s="11"/>
     </row>
-    <row r="75" ht="13.85" spans="1:3">
+    <row r="75" ht="16.8" spans="1:3">
       <c r="A75" s="12" t="s">
-        <v>451</v>
+        <v>330</v>
       </c>
       <c r="B75" s="11" t="s">
-        <v>452</v>
+        <v>331</v>
       </c>
       <c r="C75" s="11">
         <v>0</v>
       </c>
     </row>
-    <row r="76" ht="13.85" spans="1:3">
+    <row r="76" ht="16.8" spans="1:3">
       <c r="A76" s="12" t="s">
-        <v>453</v>
+        <v>332</v>
       </c>
       <c r="B76" s="11" t="s">
-        <v>452</v>
+        <v>331</v>
       </c>
       <c r="C76" s="11">
         <v>1</v>
       </c>
     </row>
-    <row r="77" ht="13.85" spans="1:3">
+    <row r="77" ht="16.8" spans="1:3">
       <c r="A77" s="12" t="s">
-        <v>454</v>
+        <v>333</v>
       </c>
       <c r="B77" s="11" t="s">
-        <v>452</v>
+        <v>331</v>
       </c>
       <c r="C77" s="11">
         <v>2</v>
       </c>
     </row>
-    <row r="78" ht="13.85" spans="1:3">
+    <row r="78" ht="16.8" spans="1:3">
       <c r="A78" s="12" t="s">
-        <v>455</v>
+        <v>334</v>
       </c>
       <c r="B78" s="11" t="s">
-        <v>452</v>
+        <v>331</v>
       </c>
       <c r="C78" s="11">
         <v>3</v>
       </c>
     </row>
-    <row r="79" ht="13.85" spans="1:3">
+    <row r="79" ht="16.8" spans="1:3">
       <c r="A79" s="12" t="s">
-        <v>456</v>
+        <v>335</v>
       </c>
       <c r="B79" s="11" t="s">
-        <v>452</v>
+        <v>331</v>
       </c>
       <c r="C79" s="11">
         <v>4</v>
       </c>
     </row>
-    <row r="80" ht="13.85" spans="1:3">
+    <row r="80" ht="16.8" spans="1:3">
       <c r="A80" s="12" t="s">
-        <v>457</v>
+        <v>336</v>
       </c>
       <c r="B80" s="11" t="s">
-        <v>452</v>
+        <v>331</v>
       </c>
       <c r="C80" s="11">
         <v>5</v>
       </c>
     </row>
-    <row r="81" ht="13.85" spans="1:3">
+    <row r="81" ht="16.8" spans="1:3">
       <c r="A81" s="12" t="s">
-        <v>458</v>
+        <v>337</v>
       </c>
       <c r="B81" s="11" t="s">
-        <v>452</v>
+        <v>331</v>
       </c>
       <c r="C81" s="11">
         <v>6</v>
       </c>
     </row>
-    <row r="82" ht="13.85" spans="1:3">
+    <row r="82" ht="16.8" spans="1:3">
       <c r="A82" s="12" t="s">
-        <v>459</v>
+        <v>338</v>
       </c>
       <c r="B82" s="11" t="s">
-        <v>452</v>
+        <v>331</v>
       </c>
       <c r="C82" s="11">
         <v>7</v>
       </c>
     </row>
-    <row r="83" ht="13.85" spans="1:3">
+    <row r="83" ht="16.8" spans="1:3">
       <c r="A83" s="12" t="s">
-        <v>460</v>
+        <v>339</v>
       </c>
       <c r="B83" s="11" t="s">
-        <v>452</v>
+        <v>331</v>
       </c>
       <c r="C83" s="11">
         <v>8</v>
       </c>
     </row>
-    <row r="84" ht="13.85" spans="1:3">
+    <row r="84" ht="16.8" spans="1:3">
       <c r="A84" s="12" t="s">
-        <v>461</v>
+        <v>340</v>
       </c>
       <c r="B84" s="11" t="s">
-        <v>452</v>
+        <v>331</v>
       </c>
       <c r="C84" s="11">
         <v>9</v>
       </c>
     </row>
-    <row r="85" ht="13.85" spans="1:3">
+    <row r="85" ht="16.8" spans="1:3">
       <c r="A85" s="12" t="s">
-        <v>462</v>
+        <v>341</v>
       </c>
       <c r="B85" s="11" t="s">
-        <v>452</v>
+        <v>331</v>
       </c>
       <c r="C85" s="11">
         <v>10</v>
       </c>
     </row>
-    <row r="86" ht="13.85" spans="1:3">
+    <row r="86" ht="16.8" spans="1:3">
       <c r="A86" s="12" t="s">
-        <v>463</v>
+        <v>342</v>
       </c>
       <c r="B86" s="11" t="s">
-        <v>452</v>
+        <v>331</v>
       </c>
       <c r="C86" s="11">
         <v>11</v>
       </c>
     </row>
-    <row r="87" ht="13.85" spans="1:3">
+    <row r="87" ht="16.8" spans="1:3">
       <c r="A87" s="12" t="s">
-        <v>464</v>
+        <v>343</v>
       </c>
       <c r="B87" s="11" t="s">
-        <v>452</v>
+        <v>331</v>
       </c>
       <c r="C87" s="11">
         <v>12</v>
       </c>
     </row>
-    <row r="88" ht="13.85" spans="1:3">
+    <row r="88" ht="16.8" spans="1:3">
       <c r="A88" s="12" t="s">
-        <v>465</v>
+        <v>344</v>
       </c>
       <c r="B88" s="11" t="s">
-        <v>452</v>
+        <v>331</v>
       </c>
       <c r="C88" s="11">
         <v>13</v>
       </c>
     </row>
-    <row r="89" ht="13.85" spans="1:3">
+    <row r="89" ht="16.8" spans="1:3">
       <c r="A89" s="12" t="s">
-        <v>466</v>
+        <v>345</v>
       </c>
       <c r="B89" s="11" t="s">
-        <v>452</v>
+        <v>331</v>
       </c>
       <c r="C89" s="11">
         <v>14</v>
       </c>
     </row>
-    <row r="90" ht="13.85" spans="1:3">
+    <row r="90" ht="16.8" spans="1:3">
       <c r="A90" s="12" t="s">
-        <v>467</v>
+        <v>346</v>
       </c>
       <c r="B90" s="11" t="s">
-        <v>452</v>
+        <v>331</v>
       </c>
       <c r="C90" s="11">
         <v>15</v>
@@ -8373,155 +7655,155 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="H4:N16"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.2"/>
   <sheetData>
     <row r="4" spans="8:14">
       <c r="H4" s="1" t="s">
-        <v>468</v>
+        <v>347</v>
       </c>
       <c r="I4" s="4"/>
       <c r="J4" s="4" t="s">
-        <v>469</v>
+        <v>348</v>
       </c>
       <c r="K4" s="4"/>
       <c r="L4" s="4" t="s">
-        <v>470</v>
+        <v>349</v>
       </c>
       <c r="M4" s="4"/>
-      <c r="N4" s="5" t="s">
-        <v>471</v>
+      <c r="N4" s="7" t="s">
+        <v>350</v>
       </c>
     </row>
     <row r="5" spans="8:14">
       <c r="H5" s="2"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="6"/>
-      <c r="N5" s="7"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="8"/>
     </row>
     <row r="6" spans="8:14">
       <c r="H6" s="2"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
-      <c r="N6" s="7"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="5"/>
+      <c r="N6" s="8"/>
     </row>
     <row r="7" spans="8:14">
       <c r="H7" s="2"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
-      <c r="N7" s="7"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
+      <c r="N7" s="8"/>
     </row>
     <row r="8" spans="8:14">
       <c r="H8" s="2" t="s">
-        <v>472</v>
-      </c>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6" t="s">
-        <v>473</v>
-      </c>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6" t="s">
-        <v>474</v>
-      </c>
-      <c r="M8" s="6"/>
-      <c r="N8" s="7" t="s">
-        <v>475</v>
+        <v>351</v>
+      </c>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="M8" s="5"/>
+      <c r="N8" s="8" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="9" spans="8:14">
       <c r="H9" s="2"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
-      <c r="N9" s="7"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="8"/>
     </row>
     <row r="10" spans="8:14">
       <c r="H10" s="2"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
-      <c r="N10" s="7"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="8"/>
     </row>
     <row r="11" spans="8:14">
       <c r="H11" s="2"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="7"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+      <c r="L11" s="5"/>
+      <c r="M11" s="5"/>
+      <c r="N11" s="8"/>
     </row>
     <row r="12" spans="8:14">
       <c r="H12" s="2" t="s">
-        <v>476</v>
-      </c>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6" t="s">
-        <v>477</v>
-      </c>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6" t="s">
-        <v>478</v>
-      </c>
-      <c r="M12" s="6"/>
-      <c r="N12" s="7" t="s">
-        <v>479</v>
+        <v>355</v>
+      </c>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5" t="s">
+        <v>356</v>
+      </c>
+      <c r="K12" s="5"/>
+      <c r="L12" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="M12" s="5"/>
+      <c r="N12" s="8" t="s">
+        <v>358</v>
       </c>
     </row>
     <row r="13" spans="8:14">
       <c r="H13" s="2"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
-      <c r="N13" s="7"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="8"/>
     </row>
     <row r="14" spans="8:14">
       <c r="H14" s="2"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="6"/>
-      <c r="M14" s="6"/>
-      <c r="N14" s="7"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="8"/>
     </row>
     <row r="15" spans="8:14">
       <c r="H15" s="2"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="6"/>
-      <c r="M15" s="6"/>
-      <c r="N15" s="7"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+      <c r="L15" s="5"/>
+      <c r="M15" s="5"/>
+      <c r="N15" s="8"/>
     </row>
     <row r="16" spans="8:14">
       <c r="H16" s="3" t="s">
-        <v>480</v>
-      </c>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8" t="s">
-        <v>481</v>
-      </c>
-      <c r="K16" s="8"/>
-      <c r="L16" s="8" t="s">
-        <v>482</v>
-      </c>
-      <c r="M16" s="8"/>
+        <v>359</v>
+      </c>
+      <c r="I16" s="6"/>
+      <c r="J16" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="K16" s="6"/>
+      <c r="L16" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="M16" s="6"/>
       <c r="N16" s="9" t="s">
-        <v>483</v>
+        <v>362</v>
       </c>
     </row>
   </sheetData>

</xml_diff>